<commit_message>
fix: tipo_cliente como ID numérico en plantilla Effi
- Agrega TIPO_CLIENTE_MAP (Común=1, Fiel=2, Desertor=3, Mayorista=4, Importador=5, Industrial=6)
- Effi requiere entero en columna 'Tipo de cliente *' — antes enviaba texto y fallaba
- XLSX de prueba regenerado con los 4 valores correctos

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import_clientes_effi_TEST_2026-03-10.xlsx
+++ b/import_clientes_effi_TEST_2026-03-10.xlsx
@@ -631,10 +631,8 @@
       <c r="S2" t="n">
         <v>5</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Común</t>
-        </is>
+      <c r="T2" t="n">
+        <v>1</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -696,10 +694,8 @@
       <c r="S3" t="n">
         <v>4</v>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Mayorista</t>
-        </is>
+      <c r="T3" t="n">
+        <v>4</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -761,10 +757,8 @@
       <c r="S4" t="n">
         <v>5</v>
       </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Fiel</t>
-        </is>
+      <c r="T4" t="n">
+        <v>2</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -826,10 +820,8 @@
       <c r="S5" t="n">
         <v>4</v>
       </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Importador</t>
-        </is>
+      <c r="T5" t="n">
+        <v>5</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>

</xml_diff>